<commit_message>
updated onging research excel, publications tab in home, outreaach css
</commit_message>
<xml_diff>
--- a/excels/Research.xlsx
+++ b/excels/Research.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54995595-8062-4994-8CCE-8230C201FB3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D22B51BB-3B8D-4670-A29C-B6286DFC62B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="81">
   <si>
     <t>S.No.</t>
   </si>
@@ -256,157 +256,19 @@
     <t>Project_Title</t>
   </si>
   <si>
-    <t>Research_Domain</t>
-  </si>
-  <si>
-    <t>Technology_Used</t>
-  </si>
-  <si>
     <t>Start_Date</t>
   </si>
   <si>
-    <t>Current_Status</t>
-  </si>
-  <si>
-    <t>Completion_Percentage</t>
-  </si>
-  <si>
-    <t>Team_Size</t>
-  </si>
-  <si>
-    <t>Funding_Amount_USD</t>
-  </si>
-  <si>
-    <t>AI-Based Crop Disease Detection</t>
-  </si>
-  <si>
-    <t>Artificial Intelligence</t>
-  </si>
-  <si>
-    <t>YOLOv8, CNN</t>
-  </si>
-  <si>
-    <t>2025-02-08</t>
-  </si>
-  <si>
-    <t>Data Collection</t>
-  </si>
-  <si>
-    <t>Smart Traffic Monitoring</t>
-  </si>
-  <si>
-    <t>Computer Vision</t>
-  </si>
-  <si>
-    <t>YOLOv8, DeepSORT</t>
-  </si>
-  <si>
-    <t>2025-06-27</t>
-  </si>
-  <si>
-    <t>Development</t>
-  </si>
-  <si>
-    <t>Blockchain Voting System</t>
-  </si>
-  <si>
-    <t>Cyber Security</t>
-  </si>
-  <si>
-    <t>Ethereum, Solidity</t>
-  </si>
-  <si>
-    <t>2025-08-23</t>
-  </si>
-  <si>
-    <t>Deployment</t>
-  </si>
-  <si>
-    <t>IoT Smart Home Automation</t>
-  </si>
-  <si>
-    <t>Internet of Things</t>
-  </si>
-  <si>
-    <t>ESP32, MQTT</t>
-  </si>
-  <si>
-    <t>2025-09-03</t>
-  </si>
-  <si>
-    <t>Healthcare Chatbot</t>
-  </si>
-  <si>
-    <t>Natural Language Processing</t>
-  </si>
-  <si>
-    <t>Transformers, Python</t>
-  </si>
-  <si>
-    <t>2025-07-10</t>
-  </si>
-  <si>
-    <t>Autonomous Delivery Robot</t>
-  </si>
-  <si>
-    <t>Robotics</t>
-  </si>
-  <si>
-    <t>ROS, LiDAR</t>
-  </si>
-  <si>
-    <t>2025-12-18</t>
-  </si>
-  <si>
-    <t>Planning</t>
-  </si>
-  <si>
-    <t>Fake News Detection</t>
-  </si>
-  <si>
-    <t>Machine Learning</t>
-  </si>
-  <si>
-    <t>BERT, NLP</t>
-  </si>
-  <si>
-    <t>2025-09-17</t>
-  </si>
-  <si>
-    <t>Renewable Energy Prediction</t>
-  </si>
-  <si>
-    <t>Data Science</t>
-  </si>
-  <si>
-    <t>LSTM, TensorFlow</t>
-  </si>
-  <si>
-    <t>2025-12-17</t>
-  </si>
-  <si>
-    <t>AR Interior Design App</t>
-  </si>
-  <si>
-    <t>Augmented Reality</t>
-  </si>
-  <si>
-    <t>Unity, ARCore</t>
-  </si>
-  <si>
-    <t>2025-03-29</t>
-  </si>
-  <si>
-    <t>Student Performance Analysis</t>
-  </si>
-  <si>
-    <t>Educational Analytics</t>
-  </si>
-  <si>
-    <t>Python, Pandas</t>
-  </si>
-  <si>
-    <t>2025-09-28</t>
+    <t>Funding_amount</t>
+  </si>
+  <si>
+    <t>Funding_agency</t>
+  </si>
+  <si>
+    <t>PI&amp;CoPIs</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -763,285 +625,189 @@
         <v>75</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>82</v>
-      </c>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D2" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="E2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F2">
-        <v>94</v>
-      </c>
-      <c r="G2">
-        <v>3</v>
-      </c>
-      <c r="H2">
-        <v>12833</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="D3" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="E3" t="s">
-        <v>92</v>
-      </c>
-      <c r="F3">
-        <v>47</v>
-      </c>
-      <c r="G3">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>35013</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="D4" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="E4" t="s">
-        <v>97</v>
-      </c>
-      <c r="F4">
-        <v>92</v>
-      </c>
-      <c r="G4">
-        <v>7</v>
-      </c>
-      <c r="H4">
-        <v>34910</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="D5" t="s">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="E5" t="s">
-        <v>97</v>
-      </c>
-      <c r="F5">
-        <v>46</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>31756</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="B6" t="s">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="C6" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D6" t="s">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="E6" t="s">
-        <v>97</v>
-      </c>
-      <c r="F6">
-        <v>92</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>5826</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>106</v>
+        <v>80</v>
       </c>
       <c r="B7" t="s">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="C7" t="s">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="D7" t="s">
-        <v>109</v>
+        <v>80</v>
       </c>
       <c r="E7" t="s">
-        <v>110</v>
-      </c>
-      <c r="F7">
-        <v>52</v>
-      </c>
-      <c r="G7">
-        <v>7</v>
-      </c>
-      <c r="H7">
-        <v>19428</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>111</v>
+        <v>80</v>
       </c>
       <c r="B8" t="s">
-        <v>112</v>
+        <v>80</v>
       </c>
       <c r="C8" t="s">
-        <v>113</v>
+        <v>80</v>
       </c>
       <c r="D8" t="s">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="E8" t="s">
-        <v>97</v>
-      </c>
-      <c r="F8">
-        <v>21</v>
-      </c>
-      <c r="G8">
-        <v>2</v>
-      </c>
-      <c r="H8">
-        <v>32061</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="B9" t="s">
-        <v>116</v>
+        <v>80</v>
       </c>
       <c r="C9" t="s">
-        <v>117</v>
+        <v>80</v>
       </c>
       <c r="D9" t="s">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="E9" t="s">
-        <v>92</v>
-      </c>
-      <c r="F9">
-        <v>80</v>
-      </c>
-      <c r="G9">
-        <v>9</v>
-      </c>
-      <c r="H9">
-        <v>5932</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="B10" t="s">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="C10" t="s">
-        <v>121</v>
+        <v>80</v>
       </c>
       <c r="D10" t="s">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="E10" t="s">
-        <v>110</v>
-      </c>
-      <c r="F10">
-        <v>31</v>
-      </c>
-      <c r="G10">
-        <v>6</v>
-      </c>
-      <c r="H10">
-        <v>27967</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>123</v>
+        <v>80</v>
       </c>
       <c r="B11" t="s">
-        <v>124</v>
+        <v>80</v>
       </c>
       <c r="C11" t="s">
-        <v>125</v>
+        <v>80</v>
       </c>
       <c r="D11" t="s">
-        <v>126</v>
+        <v>80</v>
       </c>
       <c r="E11" t="s">
-        <v>97</v>
-      </c>
-      <c r="F11">
-        <v>73</v>
-      </c>
-      <c r="G11">
-        <v>4</v>
-      </c>
-      <c r="H11">
-        <v>48599</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
students data update and faculty css update
</commit_message>
<xml_diff>
--- a/excels/Research.xlsx
+++ b/excels/Research.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{069B4D0F-B904-4908-9E2F-F29D9A8370A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53A6567A-61FF-4CEE-B788-B70E0569E844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -295,13 +295,13 @@
     <t>Indian Academy of Highway Engineers (IAHE), MoRTH</t>
   </si>
   <si>
-    <t>Prof. B Raghuram Kadali, Prof. C. S. R. K. Prasad, Prof. K. V. R. Ravi Shankar</t>
-  </si>
-  <si>
     <t>Prof. K. V. R. Ravi Shankar, Prof. B Raghuram Kadali</t>
   </si>
   <si>
-    <t>Prof. B Raghuram Kadali, Prof. C. S. R. K. Prasad, Prof. K. V. R. Ravi Shankar, Prof. Arpan Mehar</t>
+    <t>Prof. C. S. R. K. Prasad, Prof. B Raghuram Kadali, Prof. K. V. R. Ravi Shankar</t>
+  </si>
+  <si>
+    <t>Prof. C. S. R. K. Prasad, Prof. B Raghuram Kadali, Prof. K. V. R. Ravi Shankar, Prof. Arpan Mehar</t>
   </si>
 </sst>
 </file>
@@ -688,7 +688,7 @@
         <v>45809</v>
       </c>
       <c r="E2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -705,7 +705,7 @@
         <v>45383</v>
       </c>
       <c r="E3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>